<commit_message>
Adding graph and datastructure
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -5,25 +5,26 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rajitha/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rajitha/testng-DSAlgo/dsalgo-testng-framework/src/test/resources/testdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77C4DBE1-EFC1-D047-A502-40B7CEC64636}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C940C1B-7511-5740-89B4-73600C290388}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="44800" windowHeight="23060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="44800" windowHeight="23060" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="dropdown" sheetId="11" r:id="rId1"/>
     <sheet name="SignIn" sheetId="2" r:id="rId2"/>
     <sheet name="Register" sheetId="3" r:id="rId3"/>
     <sheet name="Queue" sheetId="4" r:id="rId4"/>
-    <sheet name="Tree" sheetId="5" r:id="rId5"/>
-    <sheet name="CodeEditor" sheetId="6" r:id="rId6"/>
-    <sheet name="Arrays" sheetId="7" r:id="rId7"/>
-    <sheet name="Stack" sheetId="13" r:id="rId8"/>
-    <sheet name="LinkedList" sheetId="14" r:id="rId9"/>
-    <sheet name="PythonCode" sheetId="10" r:id="rId10"/>
-    <sheet name="Arrays_Practice_Editor" sheetId="12" r:id="rId11"/>
+    <sheet name="Try Here" sheetId="15" r:id="rId5"/>
+    <sheet name="Tree" sheetId="5" r:id="rId6"/>
+    <sheet name="CodeEditor" sheetId="6" r:id="rId7"/>
+    <sheet name="Arrays" sheetId="7" r:id="rId8"/>
+    <sheet name="Stack" sheetId="13" r:id="rId9"/>
+    <sheet name="LinkedList" sheetId="14" r:id="rId10"/>
+    <sheet name="PythonCode" sheetId="10" r:id="rId11"/>
+    <sheet name="Arrays_Practice_Editor" sheetId="12" r:id="rId12"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -46,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="145">
   <si>
     <t>Data Structure</t>
   </si>
@@ -514,12 +515,27 @@
     return sorted_squares_list;
 sortedSquares([-7,-3,2,3,11])</t>
   </si>
+  <si>
+    <t>Execute</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Alert</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>SyntaxError: bad input on line 1</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -566,6 +582,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -593,7 +616,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -610,6 +633,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -882,12 +906,90 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79DCABC4-BCC9-432D-ADC9-663D639FBD68}">
+  <dimension ref="A1:A13"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13"/>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" s="9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" s="9" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" s="9" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
+      <c r="A4" s="9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" s="9" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1">
+      <c r="A6" s="9" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1">
+      <c r="A7" s="9" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1">
+      <c r="A8" s="9" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1">
+      <c r="A9" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1">
+      <c r="A10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1">
+      <c r="A11" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1">
+      <c r="A12" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1">
+      <c r="A13" t="s">
+        <v>68</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:B133"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col min="1" max="1" width="28.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
@@ -917,7 +1019,7 @@
       <c r="A4" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="11" t="s">
         <v>75</v>
       </c>
     </row>
@@ -925,19 +1027,19 @@
       <c r="A5" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="B5" s="11"/>
+      <c r="B5" s="12"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="B6" s="11"/>
+      <c r="B6" s="12"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="11" t="s">
         <v>78</v>
       </c>
     </row>
@@ -945,19 +1047,19 @@
       <c r="A8" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="B8" s="11"/>
+      <c r="B8" s="12"/>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="B9" s="11"/>
+      <c r="B9" s="12"/>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="11" t="s">
         <v>81</v>
       </c>
     </row>
@@ -965,19 +1067,19 @@
       <c r="A11" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="B11" s="11"/>
+      <c r="B11" s="12"/>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="B12" s="11"/>
+      <c r="B12" s="12"/>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="11" t="s">
         <v>83</v>
       </c>
     </row>
@@ -985,19 +1087,19 @@
       <c r="A14" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="B14" s="11"/>
+      <c r="B14" s="12"/>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="B15" s="11"/>
+      <c r="B15" s="12"/>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="11" t="s">
         <v>86</v>
       </c>
     </row>
@@ -1005,19 +1107,19 @@
       <c r="A17" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="B17" s="11"/>
+      <c r="B17" s="12"/>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="B18" s="11"/>
+      <c r="B18" s="12"/>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="B19" s="10" t="s">
+      <c r="B19" s="11" t="s">
         <v>89</v>
       </c>
     </row>
@@ -1025,19 +1127,19 @@
       <c r="A20" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="B20" s="11"/>
+      <c r="B20" s="12"/>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B21" s="11"/>
+      <c r="B21" s="12"/>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="B22" s="10" t="s">
+      <c r="B22" s="11" t="s">
         <v>92</v>
       </c>
     </row>
@@ -1045,73 +1147,73 @@
       <c r="A23" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="B23" s="11"/>
+      <c r="B23" s="12"/>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="B24" s="11"/>
+      <c r="B24" s="12"/>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B25" s="11"/>
+      <c r="B25" s="12"/>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B26" s="11"/>
+      <c r="B26" s="12"/>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="B27" s="11"/>
+      <c r="B27" s="12"/>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="B28" s="11"/>
+      <c r="B28" s="12"/>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B29" s="11"/>
+      <c r="B29" s="12"/>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B30" s="11"/>
+      <c r="B30" s="12"/>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B31" s="11"/>
+      <c r="B31" s="12"/>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B32" s="11"/>
+      <c r="B32" s="12"/>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="B33" s="11"/>
+      <c r="B33" s="12"/>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="B34" s="10" t="s">
+      <c r="B34" s="11" t="s">
         <v>99</v>
       </c>
     </row>
@@ -1119,73 +1221,73 @@
       <c r="A35" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="B35" s="11"/>
+      <c r="B35" s="12"/>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="B36" s="11"/>
+      <c r="B36" s="12"/>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B37" s="11"/>
+      <c r="B37" s="12"/>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B38" s="11"/>
+      <c r="B38" s="12"/>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="B39" s="11"/>
+      <c r="B39" s="12"/>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="B40" s="11"/>
+      <c r="B40" s="12"/>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B41" s="11"/>
+      <c r="B41" s="12"/>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B42" s="11"/>
+      <c r="B42" s="12"/>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B43" s="11"/>
+      <c r="B43" s="12"/>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B44" s="11"/>
+      <c r="B44" s="12"/>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="B45" s="11"/>
+      <c r="B45" s="12"/>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="B46" s="12">
+      <c r="B46" s="13">
         <v>2</v>
       </c>
     </row>
@@ -1193,115 +1295,115 @@
       <c r="A47" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="B47" s="11"/>
+      <c r="B47" s="12"/>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="B48" s="11"/>
+      <c r="B48" s="12"/>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="B49" s="11"/>
+      <c r="B49" s="12"/>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="B50" s="11"/>
+      <c r="B50" s="12"/>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="B51" s="11"/>
+      <c r="B51" s="12"/>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B52" s="11"/>
+      <c r="B52" s="12"/>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B53" s="11"/>
+      <c r="B53" s="12"/>
     </row>
     <row r="54" spans="1:2">
       <c r="A54" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="B54" s="11"/>
+      <c r="B54" s="12"/>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="B55" s="11"/>
+      <c r="B55" s="12"/>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B56" s="11"/>
+      <c r="B56" s="12"/>
     </row>
     <row r="57" spans="1:2">
       <c r="A57" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B57" s="11"/>
+      <c r="B57" s="12"/>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="B58" s="11"/>
+      <c r="B58" s="12"/>
     </row>
     <row r="59" spans="1:2">
       <c r="A59" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B59" s="11"/>
+      <c r="B59" s="12"/>
     </row>
     <row r="60" spans="1:2">
       <c r="A60" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B60" s="11"/>
+      <c r="B60" s="12"/>
     </row>
     <row r="61" spans="1:2">
       <c r="A61" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="B61" s="11"/>
+      <c r="B61" s="12"/>
     </row>
     <row r="62" spans="1:2">
       <c r="A62" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B62" s="11"/>
+      <c r="B62" s="12"/>
     </row>
     <row r="63" spans="1:2">
       <c r="A63" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B63" s="11"/>
+      <c r="B63" s="12"/>
     </row>
     <row r="64" spans="1:2">
       <c r="A64" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="B64" s="11"/>
+      <c r="B64" s="12"/>
     </row>
     <row r="65" spans="1:2">
       <c r="A65" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="B65" s="10" t="s">
+      <c r="B65" s="11" t="s">
         <v>99</v>
       </c>
     </row>
@@ -1309,115 +1411,115 @@
       <c r="A66" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="B66" s="11"/>
+      <c r="B66" s="12"/>
     </row>
     <row r="67" spans="1:2">
       <c r="A67" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="B67" s="11"/>
+      <c r="B67" s="12"/>
     </row>
     <row r="68" spans="1:2">
       <c r="A68" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="B68" s="11"/>
+      <c r="B68" s="12"/>
     </row>
     <row r="69" spans="1:2">
       <c r="A69" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="B69" s="11"/>
+      <c r="B69" s="12"/>
     </row>
     <row r="70" spans="1:2">
       <c r="A70" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="B70" s="11"/>
+      <c r="B70" s="12"/>
     </row>
     <row r="71" spans="1:2">
       <c r="A71" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B71" s="11"/>
+      <c r="B71" s="12"/>
     </row>
     <row r="72" spans="1:2">
       <c r="A72" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B72" s="11"/>
+      <c r="B72" s="12"/>
     </row>
     <row r="73" spans="1:2">
       <c r="A73" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="B73" s="11"/>
+      <c r="B73" s="12"/>
     </row>
     <row r="74" spans="1:2">
       <c r="A74" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="B74" s="11"/>
+      <c r="B74" s="12"/>
     </row>
     <row r="75" spans="1:2">
       <c r="A75" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B75" s="11"/>
+      <c r="B75" s="12"/>
     </row>
     <row r="76" spans="1:2">
       <c r="A76" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B76" s="11"/>
+      <c r="B76" s="12"/>
     </row>
     <row r="77" spans="1:2">
       <c r="A77" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="B77" s="11"/>
+      <c r="B77" s="12"/>
     </row>
     <row r="78" spans="1:2">
       <c r="A78" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B78" s="11"/>
+      <c r="B78" s="12"/>
     </row>
     <row r="79" spans="1:2">
       <c r="A79" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B79" s="11"/>
+      <c r="B79" s="12"/>
     </row>
     <row r="80" spans="1:2">
       <c r="A80" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="B80" s="11"/>
+      <c r="B80" s="12"/>
     </row>
     <row r="81" spans="1:2">
       <c r="A81" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B81" s="11"/>
+      <c r="B81" s="12"/>
     </row>
     <row r="82" spans="1:2">
       <c r="A82" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B82" s="11"/>
+      <c r="B82" s="12"/>
     </row>
     <row r="83" spans="1:2">
       <c r="A83" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="B83" s="11"/>
+      <c r="B83" s="12"/>
     </row>
     <row r="84" spans="1:2">
       <c r="A84" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="B84" s="12">
+      <c r="B84" s="13">
         <v>2</v>
       </c>
     </row>
@@ -1425,85 +1527,85 @@
       <c r="A85" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="B85" s="11"/>
+      <c r="B85" s="12"/>
     </row>
     <row r="86" spans="1:2">
       <c r="A86" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="B86" s="11"/>
+      <c r="B86" s="12"/>
     </row>
     <row r="87" spans="1:2">
       <c r="A87" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="B87" s="11"/>
+      <c r="B87" s="12"/>
     </row>
     <row r="88" spans="1:2">
       <c r="A88" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="B88" s="11"/>
+      <c r="B88" s="12"/>
     </row>
     <row r="89" spans="1:2">
       <c r="A89" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="B89" s="11"/>
+      <c r="B89" s="12"/>
     </row>
     <row r="90" spans="1:2">
       <c r="A90" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="B90" s="11"/>
+      <c r="B90" s="12"/>
     </row>
     <row r="91" spans="1:2">
       <c r="A91" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B91" s="11"/>
+      <c r="B91" s="12"/>
     </row>
     <row r="92" spans="1:2">
       <c r="A92" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B92" s="11"/>
+      <c r="B92" s="12"/>
     </row>
     <row r="93" spans="1:2">
       <c r="A93" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B93" s="11"/>
+      <c r="B93" s="12"/>
     </row>
     <row r="94" spans="1:2">
       <c r="A94" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B94" s="11"/>
+      <c r="B94" s="12"/>
     </row>
     <row r="95" spans="1:2">
       <c r="A95" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="B95" s="11"/>
+      <c r="B95" s="12"/>
     </row>
     <row r="96" spans="1:2">
       <c r="A96" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="B96" s="11"/>
+      <c r="B96" s="12"/>
     </row>
     <row r="97" spans="1:2">
       <c r="A97" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="B97" s="11"/>
+      <c r="B97" s="12"/>
     </row>
     <row r="98" spans="1:2">
       <c r="A98" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="B98" s="10" t="s">
+      <c r="B98" s="11" t="s">
         <v>99</v>
       </c>
     </row>
@@ -1511,85 +1613,85 @@
       <c r="A99" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="B99" s="11"/>
+      <c r="B99" s="12"/>
     </row>
     <row r="100" spans="1:2">
       <c r="A100" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="B100" s="11"/>
+      <c r="B100" s="12"/>
     </row>
     <row r="101" spans="1:2">
       <c r="A101" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="B101" s="11"/>
+      <c r="B101" s="12"/>
     </row>
     <row r="102" spans="1:2">
       <c r="A102" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="B102" s="11"/>
+      <c r="B102" s="12"/>
     </row>
     <row r="103" spans="1:2">
       <c r="A103" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="B103" s="11"/>
+      <c r="B103" s="12"/>
     </row>
     <row r="104" spans="1:2">
       <c r="A104" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="B104" s="11"/>
+      <c r="B104" s="12"/>
     </row>
     <row r="105" spans="1:2">
       <c r="A105" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B105" s="11"/>
+      <c r="B105" s="12"/>
     </row>
     <row r="106" spans="1:2">
       <c r="A106" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B106" s="11"/>
+      <c r="B106" s="12"/>
     </row>
     <row r="107" spans="1:2">
       <c r="A107" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B107" s="11"/>
+      <c r="B107" s="12"/>
     </row>
     <row r="108" spans="1:2">
       <c r="A108" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B108" s="11"/>
+      <c r="B108" s="12"/>
     </row>
     <row r="109" spans="1:2">
       <c r="A109" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="B109" s="11"/>
+      <c r="B109" s="12"/>
     </row>
     <row r="110" spans="1:2">
       <c r="A110" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="B110" s="11"/>
+      <c r="B110" s="12"/>
     </row>
     <row r="111" spans="1:2">
       <c r="A111" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="B111" s="11"/>
+      <c r="B111" s="12"/>
     </row>
     <row r="112" spans="1:2">
       <c r="A112" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="B112" s="10" t="s">
+      <c r="B112" s="11" t="s">
         <v>120</v>
       </c>
     </row>
@@ -1597,67 +1699,67 @@
       <c r="A113" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="B113" s="11"/>
+      <c r="B113" s="12"/>
     </row>
     <row r="114" spans="1:2">
       <c r="A114" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="B114" s="11"/>
+      <c r="B114" s="12"/>
     </row>
     <row r="115" spans="1:2">
       <c r="A115" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="B115" s="11"/>
+      <c r="B115" s="12"/>
     </row>
     <row r="116" spans="1:2">
       <c r="A116" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="B116" s="11"/>
+      <c r="B116" s="12"/>
     </row>
     <row r="117" spans="1:2">
       <c r="A117" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B117" s="11"/>
+      <c r="B117" s="12"/>
     </row>
     <row r="118" spans="1:2">
       <c r="A118" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B118" s="11"/>
+      <c r="B118" s="12"/>
     </row>
     <row r="119" spans="1:2">
       <c r="A119" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="B119" s="11"/>
+      <c r="B119" s="12"/>
     </row>
     <row r="120" spans="1:2">
       <c r="A120" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="B120" s="11"/>
+      <c r="B120" s="12"/>
     </row>
     <row r="121" spans="1:2">
       <c r="A121" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="B121" s="11"/>
+      <c r="B121" s="12"/>
     </row>
     <row r="122" spans="1:2">
       <c r="A122" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="B122" s="11"/>
+      <c r="B122" s="12"/>
     </row>
     <row r="123" spans="1:2">
       <c r="A123" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="B123" s="10" t="s">
+      <c r="B123" s="11" t="s">
         <v>99</v>
       </c>
     </row>
@@ -1665,61 +1767,61 @@
       <c r="A124" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="B124" s="11"/>
+      <c r="B124" s="12"/>
     </row>
     <row r="125" spans="1:2">
       <c r="A125" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="B125" s="11"/>
+      <c r="B125" s="12"/>
     </row>
     <row r="126" spans="1:2">
       <c r="A126" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="B126" s="11"/>
+      <c r="B126" s="12"/>
     </row>
     <row r="127" spans="1:2">
       <c r="A127" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="B127" s="11"/>
+      <c r="B127" s="12"/>
     </row>
     <row r="128" spans="1:2">
       <c r="A128" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B128" s="11"/>
+      <c r="B128" s="12"/>
     </row>
     <row r="129" spans="1:2">
       <c r="A129" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B129" s="11"/>
+      <c r="B129" s="12"/>
     </row>
     <row r="130" spans="1:2">
       <c r="A130" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="B130" s="11"/>
+      <c r="B130" s="12"/>
     </row>
     <row r="131" spans="1:2">
       <c r="A131" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="B131" s="11"/>
+      <c r="B131" s="12"/>
     </row>
     <row r="132" spans="1:2">
       <c r="A132" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="B132" s="11"/>
+      <c r="B132" s="12"/>
     </row>
     <row r="133" spans="1:2">
       <c r="A133" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="B133" s="11"/>
+      <c r="B133" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="14">
@@ -1742,7 +1844,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDB8416B-9243-4581-8EBF-1BB7D0382C41}">
   <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13"/>
@@ -1913,7 +2015,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1" spans="1:2" ht="15.75" customHeight="1">
@@ -1928,33 +2030,25 @@
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="1" t="s">
+    </row>
+    <row r="3" spans="1:2" ht="15.75" customHeight="1">
+      <c r="B3" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A3" s="1" t="s">
+    <row r="4" spans="1:2" ht="15.75" customHeight="1">
+      <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" ht="15.75" customHeight="1">
       <c r="B4" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="15.75" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A6" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="1" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2184,6 +2278,62 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C71C9BD-0D7A-A64B-B0D5-236EC605DE2B}">
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13"/>
+  <cols>
+    <col min="1" max="1" width="25.6640625" customWidth="1"/>
+    <col min="2" max="2" width="33.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="15">
+      <c r="A1" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="15">
+      <c r="A2" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="15">
+      <c r="A3" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>142</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -2274,7 +2424,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -2333,7 +2483,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -2379,7 +2529,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C76BAED1-CD18-4754-B13C-6D7F4100A7EF}">
   <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13"/>
@@ -2412,79 +2562,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79DCABC4-BCC9-432D-ADC9-663D639FBD68}">
-  <dimension ref="A1:A13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13"/>
-  <sheetData>
-    <row r="1" spans="1:1">
-      <c r="A1" s="9" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1">
-      <c r="A2" s="9" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1">
-      <c r="A3" s="9" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1">
-      <c r="A4" s="9" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1">
-      <c r="A5" s="9" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1">
-      <c r="A6" s="9" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1">
-      <c r="A7" s="9" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1">
-      <c r="A8" s="9" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1">
-      <c r="A9" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1">
-      <c r="A10" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1">
-      <c r="A11" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1">
-      <c r="A12" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1">
-      <c r="A13" t="s">
-        <v>68</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>